<commit_message>
updating files for improving predictions
</commit_message>
<xml_diff>
--- a/data/raw/catusita/backorder12_12.xlsx
+++ b/data/raw/catusita/backorder12_12.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\YOGA\Desktop\repositories\caa\catusita\catusita_predictions\data\raw\catusita\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\YOGA\Desktop\repositories\caa\catusita\catusita_predictions\data\backup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAE36CD7-7454-4EA5-82EB-A82375467329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A4C4CB9-B979-42CC-8721-73987ADC41BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="38">
   <si>
     <t>articulo</t>
   </si>
@@ -42,103 +42,112 @@
     <t>backorder</t>
   </si>
   <si>
-    <t>ctx-014z</t>
-  </si>
-  <si>
-    <t>ctx-060</t>
-  </si>
-  <si>
-    <t>cmts-011</t>
-  </si>
-  <si>
-    <t>cmts-012</t>
-  </si>
-  <si>
-    <t>opt-005l</t>
-  </si>
-  <si>
-    <t>opt-008l</t>
-  </si>
-  <si>
-    <t>wpt-703</t>
-  </si>
-  <si>
-    <t>wpt-711</t>
-  </si>
-  <si>
-    <t>dtx-117</t>
-  </si>
-  <si>
-    <t>opn-815</t>
-  </si>
-  <si>
     <t>opt-116</t>
   </si>
   <si>
-    <t>ckt-500au</t>
-  </si>
-  <si>
-    <t>ckt-507aa-lb</t>
-  </si>
-  <si>
-    <t>ckt-508aa</t>
-  </si>
-  <si>
-    <t>ckt-508aa-lb</t>
-  </si>
-  <si>
-    <t>cmms-005</t>
-  </si>
-  <si>
     <t>cmts-003</t>
   </si>
   <si>
-    <t>crts-016</t>
-  </si>
-  <si>
-    <t>opt-810</t>
-  </si>
-  <si>
-    <t>wpm-068va</t>
-  </si>
-  <si>
-    <t>wpn-001va</t>
-  </si>
-  <si>
-    <t>wpn-107va</t>
-  </si>
-  <si>
-    <t>wpt-165va</t>
-  </si>
-  <si>
-    <t>wpt-166va</t>
-  </si>
-  <si>
     <t>wpt-168va</t>
   </si>
   <si>
-    <t>crt-005</t>
-  </si>
-  <si>
-    <t>act-002</t>
-  </si>
-  <si>
     <t>crts-003</t>
   </si>
   <si>
     <t>ctx-170z</t>
   </si>
   <si>
-    <t>opt-010l</t>
-  </si>
-  <si>
-    <t>opt-075l</t>
-  </si>
-  <si>
-    <t>wpt-111va</t>
-  </si>
-  <si>
-    <t>wpt-746</t>
+    <t>dt-628</t>
+  </si>
+  <si>
+    <t>ctx-076</t>
+  </si>
+  <si>
+    <t>dtx-202</t>
+  </si>
+  <si>
+    <t>aat-017</t>
+  </si>
+  <si>
+    <t>dt-094l</t>
+  </si>
+  <si>
+    <t>cmt-005</t>
+  </si>
+  <si>
+    <t>aat-018</t>
+  </si>
+  <si>
+    <t>dt-036</t>
+  </si>
+  <si>
+    <t>dt-611u</t>
+  </si>
+  <si>
+    <t>opt-044</t>
+  </si>
+  <si>
+    <t>dtx-099</t>
+  </si>
+  <si>
+    <t>ctx-160a</t>
+  </si>
+  <si>
+    <t>opt-115</t>
+  </si>
+  <si>
+    <t>dtx-209a</t>
+  </si>
+  <si>
+    <t>dt-064</t>
+  </si>
+  <si>
+    <t>dtx-116</t>
+  </si>
+  <si>
+    <t>ctx-071</t>
+  </si>
+  <si>
+    <t>dtx-099l</t>
+  </si>
+  <si>
+    <t>dtx-199</t>
+  </si>
+  <si>
+    <t>dt-036v</t>
+  </si>
+  <si>
+    <t>dt-124v</t>
+  </si>
+  <si>
+    <t>dtx-232a</t>
+  </si>
+  <si>
+    <t>ctx-123</t>
+  </si>
+  <si>
+    <t>dt-123v</t>
+  </si>
+  <si>
+    <t>tks58-50k</t>
+  </si>
+  <si>
+    <t>ctx-065</t>
+  </si>
+  <si>
+    <t>ckn-500-lt</t>
+  </si>
+  <si>
+    <t>dn-047</t>
+  </si>
+  <si>
+    <t>dt-063v</t>
+  </si>
+  <si>
+    <t>dt-072</t>
+  </si>
+  <si>
+    <t>dtx-197</t>
   </si>
 </sst>
 </file>
@@ -480,387 +489,357 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="1">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>500</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1">
+        <v>7</v>
+      </c>
+      <c r="B3">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="1">
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="1">
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="1">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>408</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="1">
+        <v>11</v>
+      </c>
+      <c r="B7">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8">
         <v>8</v>
-      </c>
-      <c r="B8" s="1">
-        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="1">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="B9">
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="1">
+        <v>14</v>
+      </c>
+      <c r="B10">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" s="1">
+        <v>15</v>
+      </c>
+      <c r="B11">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" s="1">
+        <v>16</v>
+      </c>
+      <c r="B12">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" s="1">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="B13">
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14" s="1">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="B14">
+        <v>201</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>15</v>
-      </c>
-      <c r="B15" s="1">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="B15">
+        <v>300</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16" s="1">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="B16">
+        <v>501</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>17</v>
-      </c>
-      <c r="B17" s="1">
+        <v>19</v>
+      </c>
+      <c r="B17">
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18" s="1">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="B18">
+        <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>4</v>
-      </c>
-      <c r="B19" s="1">
+        <v>2</v>
+      </c>
+      <c r="B19">
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>5</v>
-      </c>
-      <c r="B20" s="1">
+        <v>21</v>
+      </c>
+      <c r="B20">
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21" s="1">
+        <v>22</v>
+      </c>
+      <c r="B21">
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>6</v>
-      </c>
-      <c r="B22" s="1">
-        <v>0</v>
+        <v>23</v>
+      </c>
+      <c r="B22">
+        <v>400</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>7</v>
-      </c>
-      <c r="B23" s="1">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="B23">
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>20</v>
-      </c>
-      <c r="B24" s="1">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="B24">
+        <v>200</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>21</v>
-      </c>
-      <c r="B25" s="1">
-        <v>0</v>
+        <v>25</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>22</v>
-      </c>
-      <c r="B26" s="1">
-        <v>0</v>
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>23</v>
-      </c>
-      <c r="B27" s="1">
+        <v>26</v>
+      </c>
+      <c r="B27">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>24</v>
-      </c>
-      <c r="B28" s="1">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="B28">
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>25</v>
-      </c>
-      <c r="B29" s="1">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="B29">
+        <v>100</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>26</v>
-      </c>
-      <c r="B30" s="1">
+        <v>27</v>
+      </c>
+      <c r="B30">
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>27</v>
-      </c>
-      <c r="B31" s="1">
-        <v>0</v>
+        <v>28</v>
+      </c>
+      <c r="B31">
+        <v>400</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>28</v>
       </c>
-      <c r="B32" s="1">
-        <v>0</v>
+      <c r="B32">
+        <v>1000</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>13</v>
-      </c>
-      <c r="B33" s="1">
+        <v>29</v>
+      </c>
+      <c r="B33">
         <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>15</v>
-      </c>
-      <c r="B34" s="1">
-        <v>0</v>
+        <v>30</v>
+      </c>
+      <c r="B34">
+        <v>3440</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>18</v>
-      </c>
-      <c r="B35" s="1">
-        <v>0</v>
+        <v>30</v>
+      </c>
+      <c r="B35">
+        <v>3000</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>4</v>
-      </c>
-      <c r="B36" s="1">
+        <v>31</v>
+      </c>
+      <c r="B36">
         <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>5</v>
-      </c>
-      <c r="B37" s="1">
-        <v>0</v>
+        <v>32</v>
+      </c>
+      <c r="B37">
+        <v>30</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>29</v>
-      </c>
-      <c r="B38" s="1">
+        <v>33</v>
+      </c>
+      <c r="B38">
         <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>19</v>
-      </c>
-      <c r="B39" s="1">
+        <v>34</v>
+      </c>
+      <c r="B39">
         <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>30</v>
-      </c>
-      <c r="B40" s="1">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="B40">
+        <v>40</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>7</v>
-      </c>
-      <c r="B41" s="1">
+        <v>35</v>
+      </c>
+      <c r="B41">
         <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>31</v>
-      </c>
-      <c r="B42" s="1">
+        <v>36</v>
+      </c>
+      <c r="B42">
         <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>32</v>
-      </c>
-      <c r="B43" s="1">
-        <v>0</v>
+        <v>37</v>
+      </c>
+      <c r="B43">
+        <v>200</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
-        <v>33</v>
-      </c>
-      <c r="B44" s="1">
-        <v>0</v>
-      </c>
+      <c r="B44" s="1"/>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>25</v>
-      </c>
-      <c r="B45" s="1">
-        <v>0</v>
-      </c>
+      <c r="B45" s="1"/>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
-        <v>26</v>
-      </c>
-      <c r="B46" s="1">
-        <v>0</v>
-      </c>
+      <c r="B46" s="1"/>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
-        <v>8</v>
-      </c>
-      <c r="B47" s="1">
-        <v>0</v>
-      </c>
+      <c r="B47" s="1"/>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A48" t="s">
-        <v>9</v>
-      </c>
-      <c r="B48" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
-        <v>34</v>
-      </c>
-      <c r="B49" s="1">
-        <v>0</v>
-      </c>
+      <c r="B48" s="1"/>
+    </row>
+    <row r="49" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B49" s="1"/>
     </row>
     <row r="1496" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B1496">
@@ -869,5 +848,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>